<commit_message>
Separate override from detection; map capabilities to records
</commit_message>
<xml_diff>
--- a/templates/supervisory-capacity-records.xlsx
+++ b/templates/supervisory-capacity-records.xlsx
@@ -281,7 +281,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -323,9 +323,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -413,6 +410,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -424,9 +424,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,145 +680,145 @@
   <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="32" customWidth="1" style="24" min="1" max="1"/>
-    <col width="15" customWidth="1" style="24" min="2" max="2"/>
-    <col width="44" customWidth="1" style="24" min="3" max="3"/>
-    <col width="50" customWidth="1" style="24" min="4" max="4"/>
+    <col width="32" customWidth="1" style="23" min="1" max="1"/>
+    <col width="15" customWidth="1" style="23" min="2" max="2"/>
+    <col width="44" customWidth="1" style="23" min="3" max="3"/>
+    <col width="50" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.25" customHeight="1" s="25">
-      <c r="A1" s="26" t="inlineStr">
+    <row r="1" ht="17.25" customHeight="1" s="24">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>Supervisory capacity — scorecard</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1" s="25">
-      <c r="A2" s="27" t="inlineStr">
+    <row r="2" ht="18" customHeight="1" s="24">
+      <c r="A2" s="26" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE — delete every value below before use.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="25">
-      <c r="A3" s="28" t="inlineStr">
+    <row r="3" ht="15" customHeight="1" s="24">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Summarises the four records. Does not replace the workpaper, which carries the scope, purpose limitation and conclusion.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="29" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="24">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Period and scope</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="25">
-      <c r="A6" s="30" t="inlineStr">
+    <row r="6" ht="30" customHeight="1" s="24">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Period</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>2026-Q3</t>
         </is>
       </c>
-      <c r="C6" s="32" t="n"/>
-      <c r="D6" s="33" t="n"/>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="25">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="C6" s="31" t="n"/>
+      <c r="D6" s="32" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1" s="24">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>Systems in scope</t>
         </is>
       </c>
-      <c r="B7" s="31" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Tier 3 cyber capability review queue</t>
         </is>
       </c>
-      <c r="C7" s="32" t="n"/>
-      <c r="D7" s="33" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1" s="25">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="32" t="n"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" s="24">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Oversight function</t>
         </is>
       </c>
-      <c r="B8" s="31" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>Safety case review; model output review</t>
         </is>
       </c>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="33" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1" s="25">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="C8" s="31" t="n"/>
+      <c r="D8" s="32" t="n"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" s="24">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Reviewer population</t>
         </is>
       </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>12 on the review roster; 2 assessed in the competence matrix</t>
-        </is>
-      </c>
-      <c r="C9" s="32" t="n"/>
-      <c r="D9" s="33" t="inlineStr">
-        <is>
-          <t>Records 01 and 02 cover a sample; record 03 covers the full roster</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1" s="25">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>12 on the review roster; 3 assessed in the competence matrix, 1 in the skill-preservation exercise</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="n"/>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>Coverage differs by record: 01 covers three, 02 covers two, 03 the full roster, 04 one</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="24">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Prepared by / date</t>
         </is>
       </c>
-      <c r="B10" s="31" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
         <is>
           <t>[name], 2026-08-20</t>
         </is>
       </c>
-      <c r="C10" s="32" t="n"/>
-      <c r="D10" s="33" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="32" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="24">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>What each record showed</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="25.5" customHeight="1" s="25">
-      <c r="A13" s="34" t="inlineStr">
+    <row r="13" ht="25.5" customHeight="1" s="24">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t>Record</t>
         </is>
       </c>
-      <c r="B13" s="34" t="inlineStr">
+      <c r="B13" s="33" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C13" s="34" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="D13" s="34" t="inlineStr">
+      <c r="D13" s="33" t="inlineStr">
         <is>
           <t>Interpretation</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="63.75" customHeight="1" s="25">
-      <c r="A14" s="30" t="inlineStr">
+    <row r="14" ht="63.75" customHeight="1" s="24">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -847,24 +844,24 @@
           </r>
         </is>
       </c>
-      <c r="B14" s="35" t="inlineStr">
+      <c r="B14" s="34" t="inlineStr">
         <is>
           <t>Qualified</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>2 of 12 assessed; 1 met the criterion, 1 not determined</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>R-02 scored 12/15 against a criterion of 12/15, but the assessment was a scheduled session with no concurrent load and the reviewer informed. Record 02 shows the operating week was not like that. Repeat under operating conditions before relying on it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="63.75" customHeight="1" s="25">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>3 of 12 assessed; 1 met the criterion, 1 not determined, 1 not met</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>R-02 scored 12/15 against a criterion of 12/15, but the assessment was a scheduled session with no concurrent load and the reviewer informed; record 02 shows the operating week was not like that. R-03 did not meet the comprehension criterion, 5 of 8 against a threshold of 6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="63.75" customHeight="1" s="24">
+      <c r="A15" s="29" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -890,24 +887,24 @@
           </r>
         </is>
       </c>
-      <c r="B15" s="36" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>R-02: 32h in week 28, longest stretch 5h, no breaks recorded</t>
         </is>
       </c>
-      <c r="D15" s="33" t="inlineStr">
+      <c r="D15" s="32" t="inlineStr">
         <is>
           <t>The operating week was heavier than the conditions R-02 was assessed under. This is why record 01 is not determined for that reviewer.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="63.75" customHeight="1" s="25">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="16" ht="63.75" customHeight="1" s="24">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -933,24 +930,24 @@
           </r>
         </is>
       </c>
-      <c r="B16" s="37" t="inlineStr">
+      <c r="B16" s="36" t="inlineStr">
         <is>
           <t>Not determined</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>11 of 60 flawed items accepted; median 82%, range 55-95% across 12 reviewers</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>First round, so the spread is a baseline rather than a finding. The two lowest results were reviewers whose time-on-task records show long unbroken stretches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="63.75" customHeight="1" s="25">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="C16" s="32" t="inlineStr">
+        <is>
+          <t>Detection median 82%, override median 78%, across 12 reviewers</t>
+        </is>
+      </c>
+      <c r="D16" s="32" t="inlineStr">
+        <is>
+          <t>First round, so both spreads are baselines. Three reviewers flagged doubt and let the item through, which is a different failure from not noticing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="63.75" customHeight="1" s="24">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -976,219 +973,219 @@
           </r>
         </is>
       </c>
-      <c r="B17" s="37" t="inlineStr">
+      <c r="B17" s="36" t="inlineStr">
         <is>
           <t>Not determined</t>
         </is>
       </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>R-01: 14/20 without the system against 17/20 with it, same case set</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>R-01 only: 14/20 without the system against 17/20 with it, same case set</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
         <is>
           <t>First exercise, no prior measurement. Establishes a starting point and shows no trend.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="29" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="24">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>Status legend — evidential strength, not quality</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" s="25">
-      <c r="A20" s="38" t="inlineStr">
+    <row r="20" ht="30" customHeight="1" s="24">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>Supported</t>
         </is>
       </c>
-      <c r="B20" s="39" t="n"/>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="B20" s="38" t="n"/>
+      <c r="C20" s="32" t="inlineStr">
         <is>
           <t>A criterion was set, met, and the conditions support the inference to operation.</t>
         </is>
       </c>
-      <c r="D20" s="32" t="n"/>
-    </row>
-    <row r="21" ht="30" customHeight="1" s="25">
-      <c r="A21" s="36" t="inlineStr">
+      <c r="D20" s="31" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="24">
+      <c r="A21" s="35" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
       </c>
-      <c r="B21" s="39" t="n"/>
-      <c r="C21" s="33" t="inlineStr">
+      <c r="B21" s="38" t="n"/>
+      <c r="C21" s="32" t="inlineStr">
         <is>
           <t>Conditions or facts captured. Not an assessment, so no verdict applies; it is context for reading the others.</t>
         </is>
       </c>
-      <c r="D21" s="32" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1" s="25">
-      <c r="A22" s="35" t="inlineStr">
+      <c r="D21" s="31" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1" s="24">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>Qualified</t>
         </is>
       </c>
-      <c r="B22" s="39" t="n"/>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="B22" s="38" t="n"/>
+      <c r="C22" s="32" t="inlineStr">
         <is>
           <t>A result exists, but something limits what it supports — conditions, population, or an open follow-up.</t>
         </is>
       </c>
-      <c r="D22" s="32" t="n"/>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="25">
-      <c r="A23" s="37" t="inlineStr">
+      <c r="D22" s="31" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="24">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Not determined</t>
         </is>
       </c>
-      <c r="B23" s="39" t="n"/>
-      <c r="C23" s="33" t="inlineStr">
+      <c r="B23" s="38" t="n"/>
+      <c r="C23" s="32" t="inlineStr">
         <is>
           <t>No conclusion available. A first-round baseline, a single observation, or an assessment that cannot bear weight.</t>
         </is>
       </c>
-      <c r="D23" s="40" t="n"/>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="25">
-      <c r="A24" s="41" t="inlineStr">
+      <c r="D23" s="39" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="24">
+      <c r="A24" s="40" t="inlineStr">
         <is>
           <t>The status describes how far the evidence goes. It is not a rating of the reviewers and not a risk score.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="25"/>
-    <row r="26" ht="30" customHeight="1" s="25">
-      <c r="A26" s="29" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="24"/>
+    <row r="26" ht="30" customHeight="1" s="24">
+      <c r="A26" s="28" t="inlineStr">
         <is>
           <t>Limits of this assessment</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n"/>
-    </row>
-    <row r="27" ht="30" customHeight="1" s="25">
-      <c r="A27" s="30" t="inlineStr">
+      <c r="B26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1" s="24">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Capabilities not assessed</t>
         </is>
       </c>
-      <c r="B27" s="31" t="inlineStr">
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>Independent judgment on novel questions</t>
         </is>
       </c>
-      <c r="C27" s="32" t="n"/>
-      <c r="D27" s="33" t="inlineStr">
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="32" t="inlineStr">
         <is>
           <t>Not assessable by these methods</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="30" customHeight="1" s="25">
-      <c r="A28" s="30" t="inlineStr">
+    <row r="28" ht="30" customHeight="1" s="24">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>Population caveat</t>
         </is>
       </c>
-      <c r="B28" s="31" t="inlineStr">
+      <c r="B28" s="30" t="inlineStr">
         <is>
           <t>Assessed under conditions unlike operation for R-02</t>
         </is>
       </c>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="33" t="n"/>
-    </row>
-    <row r="29" ht="23.85" customHeight="1" s="25">
-      <c r="A29" s="30" t="inlineStr">
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="32" t="n"/>
+    </row>
+    <row r="29" ht="23.25" customHeight="1" s="24">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>Comparison available</t>
         </is>
       </c>
-      <c r="B29" s="31" t="inlineStr">
+      <c r="B29" s="30" t="inlineStr">
         <is>
           <t>No — first round for 03 and 04</t>
         </is>
       </c>
-      <c r="C29" s="40" t="n"/>
-      <c r="D29" s="33" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="25"/>
-    <row r="31" ht="30" customHeight="1" s="25">
-      <c r="A31" s="29" t="inlineStr">
+      <c r="C29" s="39" t="n"/>
+      <c r="D29" s="32" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="24"/>
+    <row r="31" ht="30" customHeight="1" s="24">
+      <c r="A31" s="28" t="inlineStr">
         <is>
           <t>Conclusion</t>
         </is>
       </c>
-      <c r="B31" s="24" t="n"/>
-    </row>
-    <row r="32" ht="30" customHeight="1" s="25">
-      <c r="A32" s="30" t="inlineStr">
+      <c r="B31" s="23" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1" s="24">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>What this assessment supports</t>
         </is>
       </c>
-      <c r="B32" s="31" t="inlineStr">
-        <is>
-          <t>Competence criteria are now stated; 1 of 12 reviewers assessed against one and met it</t>
-        </is>
-      </c>
-      <c r="C32" s="32" t="n"/>
-      <c r="D32" s="33" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1" s="25">
-      <c r="A33" s="30" t="inlineStr">
+      <c r="B32" s="30" t="inlineStr">
+        <is>
+          <t>Competence criteria are stated for three reviewers; detection and override were measured separately across the full roster</t>
+        </is>
+      </c>
+      <c r="C32" s="31" t="n"/>
+      <c r="D32" s="32" t="n"/>
+    </row>
+    <row r="33" ht="30" customHeight="1" s="24">
+      <c r="A33" s="29" t="inlineStr">
         <is>
           <t>What it does not support</t>
         </is>
       </c>
-      <c r="B33" s="31" t="inlineStr">
+      <c r="B33" s="30" t="inlineStr">
         <is>
           <t>Any statement that oversight is operating effectively across the roster</t>
         </is>
       </c>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="33" t="n"/>
-    </row>
-    <row r="34" ht="30" customHeight="1" s="25">
-      <c r="A34" s="30" t="inlineStr">
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="32" t="n"/>
+    </row>
+    <row r="34" ht="30" customHeight="1" s="24">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>Action arising</t>
         </is>
       </c>
-      <c r="B34" s="31" t="inlineStr">
-        <is>
-          <t>Repeat R-02 under operating conditions; second stress-test round Q4</t>
-        </is>
-      </c>
-      <c r="C34" s="32" t="n"/>
-      <c r="D34" s="33" t="inlineStr">
+      <c r="B34" s="30" t="inlineStr">
+        <is>
+          <t>Remediate R-03 comprehension; repeat R-02 under operating conditions; second stress-test round Q4</t>
+        </is>
+      </c>
+      <c r="C34" s="31" t="n"/>
+      <c r="D34" s="32" t="inlineStr">
         <is>
           <t>Cross-reference the workpaper</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="25">
-      <c r="A35" s="30" t="inlineStr">
+    <row r="35" ht="15" customHeight="1" s="24">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>Workpaper reference</t>
         </is>
       </c>
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="30" t="inlineStr">
         <is>
           <t>[reference]</t>
         </is>
       </c>
-      <c r="C35" s="40" t="n"/>
-      <c r="D35" s="33" t="n"/>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="25"/>
-    <row r="37" ht="15" customHeight="1" s="25">
-      <c r="A37" s="41" t="inlineStr">
+      <c r="C35" s="39" t="n"/>
+      <c r="D35" s="32" t="n"/>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="24"/>
+    <row r="37" ht="15" customHeight="1" s="24">
+      <c r="A37" s="40" t="inlineStr">
         <is>
           <t>Not a compliance opinion. See README.md for ethics, employment obligations and disclaimer.</t>
         </is>
@@ -1224,286 +1221,373 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="24" customWidth="1" style="24" min="1" max="10"/>
-    <col width="34" customWidth="1" style="24" min="11" max="11"/>
-    <col width="24" customWidth="1" style="24" min="12" max="17"/>
+    <col width="24" customWidth="1" style="23" min="1" max="10"/>
+    <col width="34" customWidth="1" style="23" min="11" max="11"/>
+    <col width="24" customWidth="1" style="23" min="12" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="25">
-      <c r="A1" s="34" t="inlineStr">
+    <row r="1" ht="33.75" customHeight="1" s="24">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>reviewer_id</t>
         </is>
       </c>
-      <c r="B1" s="34" t="inlineStr">
+      <c r="B1" s="33" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="C1" s="34" t="inlineStr">
+      <c r="C1" s="33" t="inlineStr">
         <is>
           <t>system_scope</t>
         </is>
       </c>
-      <c r="D1" s="34" t="inlineStr">
+      <c r="D1" s="33" t="inlineStr">
         <is>
           <t>required_skill</t>
         </is>
       </c>
-      <c r="E1" s="34" t="inlineStr">
+      <c r="E1" s="33" t="inlineStr">
         <is>
           <t>required_level</t>
         </is>
       </c>
-      <c r="F1" s="34" t="inlineStr">
+      <c r="F1" s="33" t="inlineStr">
         <is>
           <t>assessment_method</t>
         </is>
       </c>
-      <c r="G1" s="34" t="inlineStr">
+      <c r="G1" s="33" t="inlineStr">
         <is>
           <t>assessment_date</t>
         </is>
       </c>
-      <c r="H1" s="34" t="inlineStr">
+      <c r="H1" s="33" t="inlineStr">
         <is>
           <t>criterion</t>
         </is>
       </c>
-      <c r="I1" s="34" t="inlineStr">
+      <c r="I1" s="33" t="inlineStr">
         <is>
           <t>result</t>
         </is>
       </c>
-      <c r="J1" s="34" t="inlineStr">
+      <c r="J1" s="33" t="inlineStr">
         <is>
           <t>result_detail</t>
         </is>
       </c>
-      <c r="K1" s="34" t="inlineStr">
+      <c r="K1" s="33" t="inlineStr">
         <is>
           <t>met</t>
         </is>
       </c>
-      <c r="L1" s="34" t="inlineStr">
+      <c r="L1" s="33" t="inlineStr">
         <is>
           <t>conditions</t>
         </is>
       </c>
-      <c r="M1" s="34" t="inlineStr">
+      <c r="M1" s="33" t="inlineStr">
         <is>
           <t>next_due_date</t>
         </is>
       </c>
-      <c r="N1" s="34" t="inlineStr">
+      <c r="N1" s="33" t="inlineStr">
         <is>
           <t>remediation</t>
         </is>
       </c>
-      <c r="O1" s="34" t="inlineStr">
+      <c r="O1" s="33" t="inlineStr">
         <is>
           <t>authority_to_halt</t>
         </is>
       </c>
-      <c r="P1" s="34" t="inlineStr">
+      <c r="P1" s="33" t="inlineStr">
         <is>
           <t>evidence_location</t>
         </is>
       </c>
-      <c r="Q1" s="34" t="inlineStr">
+      <c r="Q1" s="33" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="23.85" customHeight="1" s="25">
-      <c r="A2" s="42" t="inlineStr">
+    <row r="2" ht="23.85" customHeight="1" s="24">
+      <c r="A2" s="41" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE-01</t>
         </is>
       </c>
-      <c r="B2" s="42" t="inlineStr">
+      <c r="B2" s="41" t="inlineStr">
         <is>
           <t>Safety case reviewer</t>
         </is>
       </c>
-      <c r="C2" s="42" t="inlineStr">
+      <c r="C2" s="41" t="inlineStr">
         <is>
           <t>Cyber capability tier 3</t>
         </is>
       </c>
-      <c r="D2" s="42" t="inlineStr">
+      <c r="D2" s="41" t="inlineStr">
         <is>
           <t>Identifies an unsupported step in an exploit-chain argument</t>
         </is>
       </c>
-      <c r="E2" s="42" t="inlineStr">
+      <c r="E2" s="41" t="inlineStr">
         <is>
           <t>Expert</t>
         </is>
       </c>
-      <c r="F2" s="42" t="inlineStr">
+      <c r="F2" s="41" t="inlineStr">
         <is>
           <t>Seeded error detection, 20 cases</t>
         </is>
       </c>
-      <c r="G2" s="42" t="inlineStr">
+      <c r="G2" s="41" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="H2" s="42" t="inlineStr">
+      <c r="H2" s="41" t="inlineStr">
         <is>
           <t>17/20 or better with no miss in the first ten cases</t>
         </is>
       </c>
-      <c r="I2" s="42" t="inlineStr">
+      <c r="I2" s="41" t="inlineStr">
         <is>
           <t>17/20</t>
         </is>
       </c>
-      <c r="J2" s="42" t="inlineStr">
+      <c r="J2" s="41" t="inlineStr">
         <is>
           <t>3 missed, all in cases 15-20</t>
         </is>
       </c>
-      <c r="K2" s="43" t="inlineStr">
+      <c r="K2" s="42" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="L2" s="42" t="inlineStr">
+      <c r="L2" s="41" t="inlineStr">
         <is>
           <t>End of shift, concurrent queue, reviewer not informed</t>
         </is>
       </c>
-      <c r="M2" s="42" t="inlineStr">
+      <c r="M2" s="41" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="N2" s="42" t="inlineStr">
+      <c r="N2" s="41" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O2" s="42" t="inlineStr">
+      <c r="O2" s="41" t="inlineStr">
         <is>
           <t>Independent authority to block deployment</t>
         </is>
       </c>
-      <c r="P2" s="42" t="inlineStr">
+      <c r="P2" s="41" t="inlineStr">
         <is>
           <t>GRC record store</t>
         </is>
       </c>
-      <c r="Q2" s="42" t="inlineStr">
+      <c r="Q2" s="41" t="inlineStr">
         <is>
           <t>Current</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="35.05" customHeight="1" s="25">
-      <c r="A3" s="42" t="inlineStr">
+    <row r="3" ht="35.05" customHeight="1" s="24">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE-02</t>
         </is>
       </c>
-      <c r="B3" s="42" t="inlineStr">
+      <c r="B3" s="41" t="inlineStr">
         <is>
           <t>Model output reviewer</t>
         </is>
       </c>
-      <c r="C3" s="42" t="inlineStr">
+      <c r="C3" s="41" t="inlineStr">
         <is>
           <t>Biological capability tier 4</t>
         </is>
       </c>
-      <c r="D3" s="42" t="inlineStr">
+      <c r="D3" s="41" t="inlineStr">
         <is>
           <t>Detects a manipulated statistical result in a submitted analysis</t>
         </is>
       </c>
-      <c r="E3" s="42" t="inlineStr">
+      <c r="E3" s="41" t="inlineStr">
         <is>
           <t>Authority</t>
         </is>
       </c>
-      <c r="F3" s="42" t="inlineStr">
+      <c r="F3" s="41" t="inlineStr">
         <is>
           <t>Manipulated analysis, 15 cases</t>
         </is>
       </c>
-      <c r="G3" s="42" t="inlineStr">
+      <c r="G3" s="41" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="H3" s="42" t="inlineStr">
+      <c r="H3" s="41" t="inlineStr">
         <is>
           <t>12/15 or better; any miss on a manipulated result to be discussed</t>
         </is>
       </c>
-      <c r="I3" s="42" t="inlineStr">
+      <c r="I3" s="41" t="inlineStr">
         <is>
           <t>12/15</t>
         </is>
       </c>
-      <c r="J3" s="42" t="inlineStr">
+      <c r="J3" s="41" t="inlineStr">
         <is>
           <t>2 missed, one of them a manipulated result; 1 recorded as uncertain</t>
         </is>
       </c>
-      <c r="K3" s="43" t="inlineStr">
+      <c r="K3" s="42" t="inlineStr">
         <is>
           <t>Not determined — assessment conditions unlike operation</t>
         </is>
       </c>
-      <c r="L3" s="42" t="inlineStr">
+      <c r="L3" s="41" t="inlineStr">
         <is>
           <t>Scheduled session, no concurrent load, reviewer informed</t>
         </is>
       </c>
-      <c r="M3" s="42" t="inlineStr">
+      <c r="M3" s="41" t="inlineStr">
         <is>
           <t>2026-10-10</t>
         </is>
       </c>
-      <c r="N3" s="42" t="inlineStr">
+      <c r="N3" s="41" t="inlineStr">
         <is>
           <t>Repeat under operating conditions before next cycle</t>
         </is>
       </c>
-      <c r="O3" s="42" t="inlineStr">
+      <c r="O3" s="41" t="inlineStr">
         <is>
           <t>Independent authority to block deployment</t>
         </is>
       </c>
-      <c r="P3" s="42" t="inlineStr">
+      <c r="P3" s="41" t="inlineStr">
         <is>
           <t>GRC record store</t>
         </is>
       </c>
-      <c r="Q3" s="42" t="inlineStr">
+      <c r="Q3" s="41" t="inlineStr">
         <is>
           <t>Follow-up open</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="41" t="inlineStr">
+    <row r="4" ht="46.25" customHeight="1" s="24">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>ILLUSTRATIVE-03</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Safety case reviewer</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Cyber capability tier 3</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>Explains, without reference material, why the system produced a given output and what would change it</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>Unassisted comprehension assessment, 8 scenarios</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>Explains mechanism correctly in 6 of 8 scenarios</t>
+        </is>
+      </c>
+      <c r="I4" s="41" t="inlineStr">
+        <is>
+          <t>5/8</t>
+        </is>
+      </c>
+      <c r="J4" s="41" t="inlineStr">
+        <is>
+          <t>Two failures both on outputs involving retrieval rather than generation</t>
+        </is>
+      </c>
+      <c r="K4" s="42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L4" s="41" t="inlineStr">
+        <is>
+          <t>Scheduled, no reference material, reviewer informed</t>
+        </is>
+      </c>
+      <c r="M4" s="41" t="inlineStr">
+        <is>
+          <t>2027-01-18</t>
+        </is>
+      </c>
+      <c r="N4" s="41" t="inlineStr">
+        <is>
+          <t>Targeted briefing on retrieval behaviour; reassess in six months</t>
+        </is>
+      </c>
+      <c r="O4" s="41" t="inlineStr">
+        <is>
+          <t>Independent authority to block deployment</t>
+        </is>
+      </c>
+      <c r="P4" s="41" t="inlineStr">
+        <is>
+          <t>GRC record store</t>
+        </is>
+      </c>
+      <c r="Q4" s="41" t="inlineStr">
+        <is>
+          <t>Remediation open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="24">
+      <c r="A6" s="40" t="inlineStr">
         <is>
           <t>Set the criterion before the assessment, not after. Example rows are illustrative — delete before use.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="25">
-      <c r="A6" s="44" t="inlineStr">
-        <is>
-          <t>Shaded columns carry the judgment: whether the criterion was met, and what the row means.</t>
+    <row r="7" ht="15" customHeight="1" s="24">
+      <c r="A7" s="43" t="inlineStr">
+        <is>
+          <t>Shaded columns carry the judgment: whether the criterion was met, override behaviour, and what the row means.</t>
         </is>
       </c>
     </row>
@@ -1516,362 +1600,398 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+  <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:J6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="24" customWidth="1" style="25" min="1" max="1"/>
-    <col width="24" customWidth="1" style="25" min="2" max="2"/>
-    <col width="24" customWidth="1" style="25" min="3" max="3"/>
-    <col width="24" customWidth="1" style="25" min="4" max="4"/>
-    <col width="24" customWidth="1" style="25" min="5" max="5"/>
-    <col width="24" customWidth="1" style="25" min="6" max="6"/>
-    <col width="24" customWidth="1" style="25" min="7" max="7"/>
-    <col width="24" customWidth="1" style="25" min="8" max="8"/>
-    <col width="34" customWidth="1" style="25" min="9" max="9"/>
-    <col width="24" customWidth="1" style="25" min="10" max="10"/>
+    <col width="24" customWidth="1" style="23" min="1" max="8"/>
+    <col width="34" customWidth="1" style="23" min="9" max="9"/>
+    <col width="24" customWidth="1" style="23" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="25">
-      <c r="A1" s="45" t="inlineStr">
+    <row r="1" ht="33.75" customHeight="1" s="24">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>reviewer_id</t>
         </is>
       </c>
-      <c r="B1" s="45" t="inlineStr">
+      <c r="B1" s="33" t="inlineStr">
         <is>
           <t>period</t>
         </is>
       </c>
-      <c r="C1" s="45" t="inlineStr">
+      <c r="C1" s="33" t="inlineStr">
         <is>
           <t>items_reviewed</t>
         </is>
       </c>
-      <c r="D1" s="45" t="inlineStr">
+      <c r="D1" s="33" t="inlineStr">
         <is>
           <t>hours_total</t>
         </is>
       </c>
-      <c r="E1" s="45" t="inlineStr">
+      <c r="E1" s="33" t="inlineStr">
         <is>
           <t>longest_continuous_stretch</t>
         </is>
       </c>
-      <c r="F1" s="45" t="inlineStr">
+      <c r="F1" s="33" t="inlineStr">
         <is>
           <t>break_pattern</t>
         </is>
       </c>
-      <c r="G1" s="45" t="inlineStr">
+      <c r="G1" s="33" t="inlineStr">
         <is>
           <t>concurrent_scenarios</t>
         </is>
       </c>
-      <c r="H1" s="45" t="inlineStr">
+      <c r="H1" s="33" t="inlineStr">
         <is>
           <t>task_difficulty_note</t>
         </is>
       </c>
-      <c r="I1" s="45" t="inlineStr">
+      <c r="I1" s="33" t="inlineStr">
         <is>
           <t>interpretation</t>
         </is>
       </c>
-      <c r="J1" s="45" t="inlineStr">
+      <c r="J1" s="33" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="46" t="inlineStr">
+    <row r="2" ht="23.85" customHeight="1" s="24">
+      <c r="A2" s="41" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE-01</t>
         </is>
       </c>
-      <c r="B2" s="46" t="inlineStr">
+      <c r="B2" s="41" t="inlineStr">
         <is>
           <t>2026-W28</t>
         </is>
       </c>
-      <c r="C2" s="46" t="inlineStr">
+      <c r="C2" s="41" t="inlineStr">
         <is>
           <t>142</t>
         </is>
       </c>
-      <c r="D2" s="46" t="inlineStr">
+      <c r="D2" s="41" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="E2" s="46" t="inlineStr">
+      <c r="E2" s="41" t="inlineStr">
         <is>
           <t>1h 30m</t>
         </is>
       </c>
-      <c r="F2" s="46" t="inlineStr">
+      <c r="F2" s="41" t="inlineStr">
         <is>
           <t>15 min per 90 min</t>
         </is>
       </c>
-      <c r="G2" s="46" t="inlineStr">
+      <c r="G2" s="41" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H2" s="46" t="inlineStr">
+      <c r="H2" s="41" t="inlineStr">
         <is>
           <t>Routine cases, verification straightforward</t>
         </is>
       </c>
-      <c r="I2" s="47" t="inlineStr">
+      <c r="I2" s="42" t="inlineStr">
         <is>
           <t>Within the pattern set for this queue — 28 hours, breaks every 90 minutes.</t>
         </is>
       </c>
-      <c r="J2" s="46" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="46" t="inlineStr">
+      <c r="J2" s="41" t="n"/>
+    </row>
+    <row r="3" ht="46.25" customHeight="1" s="24">
+      <c r="A3" s="41" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE-02</t>
         </is>
       </c>
-      <c r="B3" s="46" t="inlineStr">
+      <c r="B3" s="41" t="inlineStr">
         <is>
           <t>2026-W28</t>
         </is>
       </c>
-      <c r="C3" s="46" t="inlineStr">
+      <c r="C3" s="41" t="inlineStr">
         <is>
           <t>210</t>
         </is>
       </c>
-      <c r="D3" s="46" t="inlineStr">
+      <c r="D3" s="41" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="E3" s="46" t="inlineStr">
+      <c r="E3" s="41" t="inlineStr">
         <is>
           <t>5h 00m</t>
         </is>
       </c>
-      <c r="F3" s="46" t="inlineStr">
+      <c r="F3" s="41" t="inlineStr">
         <is>
           <t>None recorded</t>
         </is>
       </c>
-      <c r="G3" s="46" t="inlineStr">
+      <c r="G3" s="41" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H3" s="46" t="inlineStr">
+      <c r="H3" s="41" t="inlineStr">
         <is>
           <t>Two cases required independent replication of a statistical result</t>
         </is>
       </c>
-      <c r="I3" s="47" t="inlineStr">
+      <c r="I3" s="42" t="inlineStr">
         <is>
           <t>32 hours with a five-hour unbroken stretch and four concurrent scenarios. Any assessment result from this week should be read with that in view.</t>
         </is>
       </c>
-      <c r="J3" s="46" t="inlineStr">
+      <c r="J3" s="41" t="inlineStr">
         <is>
           <t>Verification complexity high in two cases</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="48" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="24">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>The construct is cognitive load, not concurrency alone.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="49" t="inlineStr">
-        <is>
-          <t>Shaded columns carry the judgment: whether the criterion was met, and what the row means.</t>
+    <row r="6" ht="15" customHeight="1" s="24">
+      <c r="A6" s="43" t="inlineStr">
+        <is>
+          <t>Shaded columns carry the judgment: whether the criterion was met, override behaviour, and what the row means.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <dimension ref="A1:P5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="24" min="1" max="11"/>
-    <col width="34" customWidth="1" style="24" min="12" max="12"/>
+    <col width="24" customWidth="1" style="24" min="1" max="1"/>
+    <col width="24" customWidth="1" style="24" min="2" max="2"/>
+    <col width="24" customWidth="1" style="24" min="3" max="3"/>
+    <col width="24" customWidth="1" style="24" min="4" max="4"/>
+    <col width="24" customWidth="1" style="24" min="5" max="5"/>
+    <col width="24" customWidth="1" style="24" min="6" max="6"/>
+    <col width="24" customWidth="1" style="24" min="7" max="7"/>
+    <col width="24" customWidth="1" style="24" min="8" max="8"/>
+    <col width="24" customWidth="1" style="24" min="9" max="9"/>
+    <col width="34" customWidth="1" style="24" min="10" max="10"/>
+    <col width="34" customWidth="1" style="24" min="11" max="11"/>
+    <col width="24" customWidth="1" style="24" min="12" max="12"/>
     <col width="24" customWidth="1" style="24" min="13" max="13"/>
+    <col width="24" customWidth="1" style="24" min="14" max="14"/>
+    <col width="34" customWidth="1" style="24" min="15" max="15"/>
+    <col width="24" customWidth="1" style="24" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="25">
-      <c r="A1" s="34" t="inlineStr">
+    <row r="1" ht="34" customHeight="1" s="24">
+      <c r="A1" s="45" t="inlineStr">
         <is>
           <t>test_id</t>
         </is>
       </c>
-      <c r="B1" s="34" t="inlineStr">
+      <c r="B1" s="45" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="C1" s="34" t="inlineStr">
+      <c r="C1" s="45" t="inlineStr">
         <is>
           <t>population_tested</t>
         </is>
       </c>
-      <c r="D1" s="34" t="inlineStr">
+      <c r="D1" s="45" t="inlineStr">
         <is>
           <t>population_description</t>
         </is>
       </c>
-      <c r="E1" s="34" t="inlineStr">
+      <c r="E1" s="45" t="inlineStr">
         <is>
           <t>items_presented</t>
         </is>
       </c>
-      <c r="F1" s="34" t="inlineStr">
+      <c r="F1" s="45" t="inlineStr">
         <is>
           <t>flawed_items</t>
         </is>
       </c>
-      <c r="G1" s="34" t="inlineStr">
+      <c r="G1" s="45" t="inlineStr">
         <is>
           <t>flawed_items_accepted</t>
         </is>
       </c>
-      <c r="H1" s="34" t="inlineStr">
+      <c r="H1" s="45" t="inlineStr">
+        <is>
+          <t>system_confidence</t>
+        </is>
+      </c>
+      <c r="I1" s="45" t="inlineStr">
         <is>
           <t>detection_distribution</t>
         </is>
       </c>
-      <c r="I1" s="34" t="inlineStr">
+      <c r="J1" s="45" t="inlineStr">
+        <is>
+          <t>override_distribution</t>
+        </is>
+      </c>
+      <c r="K1" s="45" t="inlineStr">
+        <is>
+          <t>noticed_not_acted</t>
+        </is>
+      </c>
+      <c r="L1" s="45" t="inlineStr">
         <is>
           <t>reviewers_informed</t>
         </is>
       </c>
-      <c r="J1" s="34" t="inlineStr">
+      <c r="M1" s="45" t="inlineStr">
         <is>
           <t>ethics_review</t>
         </is>
       </c>
-      <c r="K1" s="34" t="inlineStr">
+      <c r="N1" s="45" t="inlineStr">
         <is>
           <t>conditions</t>
         </is>
       </c>
-      <c r="L1" s="34" t="inlineStr">
+      <c r="O1" s="45" t="inlineStr">
         <is>
           <t>interpretation</t>
         </is>
       </c>
-      <c r="M1" s="34" t="inlineStr">
+      <c r="P1" s="45" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="57.45" customHeight="1" s="25">
-      <c r="A2" s="42" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="46" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE</t>
         </is>
       </c>
-      <c r="B2" s="42" t="inlineStr">
+      <c r="B2" s="46" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="C2" s="42" t="inlineStr">
+      <c r="C2" s="46" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="D2" s="42" t="inlineStr">
+      <c r="D2" s="46" t="inlineStr">
         <is>
           <t>Full review roster, all shifts</t>
         </is>
       </c>
-      <c r="E2" s="42" t="inlineStr">
+      <c r="E2" s="46" t="inlineStr">
         <is>
           <t>240</t>
         </is>
       </c>
-      <c r="F2" s="42" t="inlineStr">
+      <c r="F2" s="46" t="inlineStr">
         <is>
           <t>60</t>
         </is>
       </c>
-      <c r="G2" s="42" t="inlineStr">
+      <c r="G2" s="46" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="H2" s="42" t="inlineStr">
+      <c r="H2" s="46" t="inlineStr">
+        <is>
+          <t>Presented as confident in all flawed cases</t>
+        </is>
+      </c>
+      <c r="I2" s="46" t="inlineStr">
         <is>
           <t>Median 82%, range 55-95%</t>
         </is>
       </c>
-      <c r="I2" s="42" t="inlineStr">
+      <c r="J2" s="47" t="inlineStr">
+        <is>
+          <t>Median 78%, range 50-95%</t>
+        </is>
+      </c>
+      <c r="K2" s="47" t="inlineStr">
+        <is>
+          <t>3 of 60: flagged doubt in the comment field and let the item through</t>
+        </is>
+      </c>
+      <c r="L2" s="46" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="J2" s="42" t="inlineStr">
+      <c r="M2" s="46" t="inlineStr">
         <is>
           <t>Design reviewed [ref]; works council notified [date]</t>
         </is>
       </c>
-      <c r="K2" s="42" t="inlineStr">
+      <c r="N2" s="46" t="inlineStr">
         <is>
           <t>Normal queue, no scheduling change, synthetic cases only</t>
         </is>
       </c>
-      <c r="L2" s="43" t="inlineStr">
-        <is>
-          <t>Median 82%, range 55-95%. The two lowest results were reviewers whose time-on-task records show long unbroken stretches. First round, so the spread is a baseline rather than a finding.</t>
-        </is>
-      </c>
-      <c r="M2" s="42" t="inlineStr">
-        <is>
-          <t>11 of 60 flawed items accepted</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="25">
-      <c r="A4" s="41" t="inlineStr">
-        <is>
-          <t>Record a distribution, not a pass rate. Seeded errors are deception — see the ethics section before running.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="44" t="inlineStr">
-        <is>
-          <t>Shaded columns carry the judgment: whether the criterion was met, and what the row means.</t>
+      <c r="O2" s="47" t="inlineStr">
+        <is>
+          <t>Detection median 82%, override median 78%. The gap is small but three reviewers flagged doubt and let the item through, which is a different failure from not noticing. First round, so both spreads are baselines.</t>
+        </is>
+      </c>
+      <c r="P2" s="46" t="inlineStr">
+        <is>
+          <t>Comment field used in 9 of 60 flawed cases</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="48" t="inlineStr">
+        <is>
+          <t>Detection and override are separate capabilities — record them separately. Seeded errors are deception; see the ethics section before running.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="49" t="inlineStr">
+        <is>
+          <t>Shaded columns carry the judgment: whether the criterion was met, override behaviour, and what the row means.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -1884,112 +2004,112 @@
   <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="24" customWidth="1" style="24" min="1" max="7"/>
-    <col width="34" customWidth="1" style="24" min="8" max="8"/>
-    <col width="24" customWidth="1" style="24" min="9" max="9"/>
+    <col width="24" customWidth="1" style="23" min="1" max="7"/>
+    <col width="34" customWidth="1" style="23" min="8" max="8"/>
+    <col width="24" customWidth="1" style="23" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="25">
-      <c r="A1" s="34" t="inlineStr">
+    <row r="1" ht="33.75" customHeight="1" s="24">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>reviewer_id</t>
         </is>
       </c>
-      <c r="B1" s="34" t="inlineStr">
+      <c r="B1" s="33" t="inlineStr">
         <is>
           <t>exercise_date</t>
         </is>
       </c>
-      <c r="C1" s="34" t="inlineStr">
+      <c r="C1" s="33" t="inlineStr">
         <is>
           <t>exercise_type</t>
         </is>
       </c>
-      <c r="D1" s="34" t="inlineStr">
+      <c r="D1" s="33" t="inlineStr">
         <is>
           <t>system_available</t>
         </is>
       </c>
-      <c r="E1" s="34" t="inlineStr">
+      <c r="E1" s="33" t="inlineStr">
         <is>
           <t>performance</t>
         </is>
       </c>
-      <c r="F1" s="34" t="inlineStr">
+      <c r="F1" s="33" t="inlineStr">
         <is>
           <t>comparison_to_assisted</t>
         </is>
       </c>
-      <c r="G1" s="34" t="inlineStr">
+      <c r="G1" s="33" t="inlineStr">
         <is>
           <t>interval_since_last</t>
         </is>
       </c>
-      <c r="H1" s="34" t="inlineStr">
+      <c r="H1" s="33" t="inlineStr">
         <is>
           <t>interpretation</t>
         </is>
       </c>
-      <c r="I1" s="34" t="inlineStr">
+      <c r="I1" s="33" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="46.25" customHeight="1" s="25">
-      <c r="A2" s="42" t="inlineStr">
+    <row r="2" ht="46.25" customHeight="1" s="24">
+      <c r="A2" s="41" t="inlineStr">
         <is>
           <t>ILLUSTRATIVE-01</t>
         </is>
       </c>
-      <c r="B2" s="42" t="inlineStr">
+      <c r="B2" s="41" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="C2" s="42" t="inlineStr">
+      <c r="C2" s="41" t="inlineStr">
         <is>
           <t>Degraded-mode exercise, usual tooling unavailable</t>
         </is>
       </c>
-      <c r="D2" s="42" t="inlineStr">
+      <c r="D2" s="41" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E2" s="42" t="inlineStr">
+      <c r="E2" s="41" t="inlineStr">
         <is>
           <t>14/20</t>
         </is>
       </c>
-      <c r="F2" s="42" t="inlineStr">
+      <c r="F2" s="41" t="inlineStr">
         <is>
           <t>Assisted 17/20 on same case set</t>
         </is>
       </c>
-      <c r="G2" s="42" t="inlineStr">
+      <c r="G2" s="41" t="inlineStr">
         <is>
           <t>None — first exercise</t>
         </is>
       </c>
-      <c r="H2" s="43" t="inlineStr">
+      <c r="H2" s="42" t="inlineStr">
         <is>
           <t>14/20 unassisted against 17/20 assisted on the same case set. Single observation with no prior measurement, so it establishes a starting point and shows no trend.</t>
         </is>
       </c>
-      <c r="I2" s="42" t="n"/>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="25">
-      <c r="A4" s="41" t="inlineStr">
+      <c r="I2" s="41" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="24">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>Assisted performance can stay high while unassisted capability declines.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="44" t="inlineStr">
-        <is>
-          <t>Shaded columns carry the judgment: whether the criterion was met, and what the row means.</t>
+    <row r="5" ht="15" customHeight="1" s="24">
+      <c r="A5" s="43" t="inlineStr">
+        <is>
+          <t>Shaded columns carry the judgment: whether the criterion was met, override behaviour, and what the row means.</t>
         </is>
       </c>
     </row>
@@ -2009,107 +2129,107 @@
   <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="112" customWidth="1" style="24" min="1" max="1"/>
+    <col width="112" customWidth="1" style="23" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="25">
-      <c r="A1" s="29" t="inlineStr">
+    <row r="1" ht="15" customHeight="1" s="24">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>Supervisory capacity assessment — templates</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="25">
-      <c r="A2" s="50" t="n"/>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="25">
-      <c r="A3" s="50" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="24">
+      <c r="A2" s="44" t="n"/>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="24">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>The four CSV files in the repository are the source of truth. The record sheets here are generated from them.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="25">
-      <c r="A4" s="50" t="inlineStr">
+    <row r="4" ht="15" customHeight="1" s="24">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>If they differ, the CSVs are correct. The scorecard is not generated and is filled by hand.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="50" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="25">
-      <c r="A6" s="50" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="24">
+      <c r="A5" s="44" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="24">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>Scorecard — the four records brought together, completed last. All values in it are illustrative.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="25">
-      <c r="A7" s="50" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="24">
+      <c r="A7" s="44" t="inlineStr">
         <is>
           <t>01 Competence matrix — can each reviewer do what the role requires? One row per reviewer per skill.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="25">
-      <c r="A8" s="50" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="24">
+      <c r="A8" s="44" t="inlineStr">
         <is>
           <t>02 Time on task — under what conditions were they working? Separates competence from workload.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="25">
-      <c r="A9" s="50" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="24">
+      <c r="A9" s="44" t="inlineStr">
         <is>
           <t>03 Oversight stress test — do they catch errors that are deliberately planted? Recorded as a distribution.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="25">
-      <c r="A10" s="50" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="24">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>04 Skill preservation — can they still do it without the system? Unassisted beside assisted.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="50" t="n"/>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="50" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="24">
+      <c r="A11" s="44" t="n"/>
+    </row>
+    <row r="12" ht="15" customHeight="1" s="24">
+      <c r="A12" s="44" t="inlineStr">
         <is>
           <t>Shaded columns on the record sheets are `met` and `interpretation`: what was concluded, and why.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="50" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="24">
+      <c r="A13" s="44" t="inlineStr">
         <is>
           <t>Not assessed by any of these: independent judgment on genuinely novel questions.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="25">
-      <c r="A14" s="50" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="24">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>All example rows are illustrative and should be deleted before use.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="50" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="50" t="inlineStr">
+    <row r="15" ht="15" customHeight="1" s="24">
+      <c r="A15" s="44" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="24">
+      <c r="A16" s="44" t="inlineStr">
         <is>
           <t>Read README.md and templates/README.md before use. Seeded-error testing is deception and</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="50" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="24">
+      <c r="A17" s="44" t="inlineStr">
         <is>
           <t>creates per-individual performance records; both carry obligations set out there.</t>
         </is>

</xml_diff>